<commit_message>
10/9 chapter0103 (5日目 10時間)
 chapter0103 70行目まで完了

BGNや暗転の修正を行いました。
</commit_message>
<xml_diff>
--- a/Assets/test260903/chapter0102.xlsx
+++ b/Assets/test260903/chapter0102.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9e870389230b728a/ドキュメント/GitHub/utageTest/Assets/test260903/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="892" documentId="11_9F6694A0EEBACB1C9082A027A8BF20B2877551EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1EE00D1B-0C75-4B7F-9699-5FF5207E4D7B}"/>
+  <xr:revisionPtr revIDLastSave="904" documentId="11_9F6694A0EEBACB1C9082A027A8BF20B2877551EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0975F838-D922-460A-9385-EF477A9512D0}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="855" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="chapter0102" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="118">
   <si>
     <t>Command</t>
   </si>
@@ -284,20 +284,6 @@
     <phoneticPr fontId="4"/>
   </si>
   <si>
-    <t>なんでか……不安でさ。
-凄く、怖いいんちゃね……</t>
-    <rPh sb="6" eb="8">
-      <t>フアン</t>
-    </rPh>
-    <rPh sb="12" eb="13">
-      <t>スゴ</t>
-    </rPh>
-    <rPh sb="15" eb="16">
-      <t>コワ</t>
-    </rPh>
-    <phoneticPr fontId="4"/>
-  </si>
-  <si>
     <t>有希の気持ちは分かるような気がする</t>
     <phoneticPr fontId="4"/>
   </si>
@@ -346,11 +332,6 @@
     <phoneticPr fontId="4"/>
   </si>
   <si>
-    <t>こんな機会滅多にない。
-普通は一生に一回もないもん</t>
-    <phoneticPr fontId="4"/>
-  </si>
-  <si>
     <t>Jump</t>
     <phoneticPr fontId="4"/>
   </si>
@@ -1062,6 +1043,30 @@
   </si>
   <si>
     <t>CharacterOff</t>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>なんでか……不安でさ。
+凄く、怖いんちゃね……</t>
+    <rPh sb="6" eb="8">
+      <t>フアン</t>
+    </rPh>
+    <rPh sb="12" eb="13">
+      <t>スゴ</t>
+    </rPh>
+    <rPh sb="15" eb="16">
+      <t>コワ</t>
+    </rPh>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>こんな機会は滅多にない。
+普通は一生に一回もないもん</t>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>頑張って、頑張って、頑張って、
+絶対に夢を叶えてくるね</t>
     <phoneticPr fontId="4"/>
   </si>
 </sst>
@@ -1378,7 +1383,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L1055"/>
+  <dimension ref="A1:L1056"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="11.44140625" customWidth="1"/>
@@ -1726,33 +1731,33 @@
         <v>26</v>
       </c>
       <c r="I31" s="9" t="s">
-        <v>55</v>
+        <v>115</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="13.5" customHeight="1">
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
       <c r="I32" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="33" spans="1:10" ht="27" customHeight="1">
       <c r="B33" s="3"/>
       <c r="I33" s="9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="34" spans="1:10" ht="27" customHeight="1">
       <c r="A34" s="3"/>
       <c r="I34" s="10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="35" spans="1:10" ht="27.6" customHeight="1">
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
       <c r="I35" s="10" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="36" spans="1:10" ht="13.5" customHeight="1">
@@ -1764,7 +1769,7 @@
       </c>
       <c r="C36" s="3"/>
       <c r="I36" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="37" spans="1:10" ht="13.5" customHeight="1">
@@ -1776,7 +1781,7 @@
       </c>
       <c r="C37" s="3"/>
       <c r="I37" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="38" spans="1:10" ht="13.5" customHeight="1">
@@ -1805,12 +1810,12 @@
         <v>26</v>
       </c>
       <c r="I40" s="10" t="s">
-        <v>62</v>
+        <v>116</v>
       </c>
     </row>
     <row r="41" spans="1:10" ht="13.5" customHeight="1">
       <c r="A41" s="3" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B41" s="3" t="s">
         <v>32</v>
@@ -1831,7 +1836,7 @@
         <v>26</v>
       </c>
       <c r="I43" s="10" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="26.4" customHeight="1">
@@ -1842,13 +1847,13 @@
         <v>26</v>
       </c>
       <c r="I44" s="10" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="J44" s="1"/>
     </row>
     <row r="45" spans="1:10" ht="13.5" customHeight="1">
       <c r="A45" s="3" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B45" s="12" t="s">
         <v>32</v>
@@ -1873,7 +1878,7 @@
         <v>26</v>
       </c>
       <c r="I47" s="10" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="J47" s="1"/>
     </row>
@@ -1881,7 +1886,7 @@
       <c r="A48" s="1"/>
       <c r="B48" s="1"/>
       <c r="I48" s="10" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="J48" s="1"/>
     </row>
@@ -1894,7 +1899,7 @@
         <v>25</v>
       </c>
       <c r="I49" s="9" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="J49" s="1"/>
     </row>
@@ -1906,7 +1911,7 @@
         <v>25</v>
       </c>
       <c r="I50" s="9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="51" spans="1:10" ht="28.8" customHeight="1">
@@ -1917,7 +1922,7 @@
         <v>26</v>
       </c>
       <c r="I51" s="9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="52" spans="1:10" ht="28.8" customHeight="1">
@@ -1929,113 +1934,114 @@
         <v>25</v>
       </c>
       <c r="I52" s="9" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10" ht="27.6" customHeight="1">
-      <c r="B53" s="12" t="s">
-        <v>24</v>
+        <v>69</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" ht="28.8" customHeight="1">
+      <c r="A53" s="1"/>
+      <c r="B53" s="13" t="s">
+        <v>23</v>
       </c>
       <c r="C53" s="13" t="s">
         <v>25</v>
       </c>
       <c r="I53" s="9" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10" ht="13.5" customHeight="1">
-      <c r="B54" s="3"/>
-      <c r="C54" s="3"/>
-      <c r="I54" s="6" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10" ht="27.6" customHeight="1">
-      <c r="A55" s="1"/>
-      <c r="B55" s="1"/>
-      <c r="I55" s="9" t="s">
-        <v>74</v>
+        <v>117</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" ht="27.6" customHeight="1">
+      <c r="B54" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C54" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="I54" s="9" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" ht="13.5" customHeight="1">
+      <c r="B55" s="3"/>
+      <c r="C55" s="3"/>
+      <c r="I55" s="6" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="56" spans="1:10" ht="27.6" customHeight="1">
       <c r="A56" s="1"/>
       <c r="B56" s="1"/>
       <c r="I56" s="9" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="57" spans="1:10" ht="27.6" customHeight="1">
-      <c r="A57" s="3"/>
+      <c r="A57" s="1"/>
       <c r="B57" s="1"/>
-      <c r="C57" s="1"/>
       <c r="I57" s="9" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="58" spans="1:10" ht="27.6" customHeight="1">
+      <c r="A58" s="3"/>
       <c r="B58" s="1"/>
       <c r="C58" s="1"/>
       <c r="I58" s="9" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" ht="27.6" customHeight="1">
+      <c r="B59" s="1"/>
+      <c r="C59" s="1"/>
+      <c r="I59" s="9" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" ht="28.2" customHeight="1">
+      <c r="B60" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="C60" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="I60" s="9" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" ht="13.5" customHeight="1">
+      <c r="A61" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B61" s="1" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="59" spans="1:10" ht="28.2" customHeight="1">
-      <c r="B59" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="C59" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="I59" s="9" t="s">
+      <c r="C61" s="1"/>
+      <c r="I61" s="6" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="60" spans="1:10" ht="13.5" customHeight="1">
-      <c r="A60" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B60" s="1" t="s">
+    <row r="62" spans="1:10" ht="13.5" customHeight="1">
+      <c r="A62" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B62" s="1"/>
+      <c r="C62" s="3"/>
+      <c r="I62" s="6"/>
+    </row>
+    <row r="63" spans="1:10" ht="13.5" customHeight="1">
+      <c r="A63" s="1"/>
+      <c r="B63" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C63" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="H63" s="1"/>
+      <c r="I63" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="C60" s="1"/>
-      <c r="I60" s="6" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="61" spans="1:10" ht="13.5" customHeight="1">
-      <c r="A61" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="B61" s="1"/>
-      <c r="C61" s="3"/>
-      <c r="I61" s="6"/>
-    </row>
-    <row r="62" spans="1:10" ht="13.5" customHeight="1">
-      <c r="A62" s="1"/>
-      <c r="B62" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C62" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="H62" s="1"/>
-      <c r="I62" s="6" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="63" spans="1:10" ht="28.2" customHeight="1">
-      <c r="A63" s="1"/>
-      <c r="B63" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="C63" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="I63" s="9" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="64" spans="1:10" ht="28.8" customHeight="1">
+    </row>
+    <row r="64" spans="1:10" ht="28.2" customHeight="1">
+      <c r="A64" s="1"/>
       <c r="B64" s="13" t="s">
         <v>23</v>
       </c>
@@ -2043,11 +2049,10 @@
         <v>26</v>
       </c>
       <c r="I64" s="9" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="65" spans="1:10" ht="27.6" customHeight="1">
-      <c r="A65" s="1"/>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" ht="28.8" customHeight="1">
       <c r="B65" s="13" t="s">
         <v>23</v>
       </c>
@@ -2055,103 +2060,103 @@
         <v>26</v>
       </c>
       <c r="I65" s="9" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="66" spans="1:10" ht="27" customHeight="1">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" ht="27.6" customHeight="1">
+      <c r="A66" s="1"/>
       <c r="B66" s="13" t="s">
         <v>23</v>
       </c>
       <c r="C66" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="H66" s="1"/>
       <c r="I66" s="9" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="67" spans="1:10" ht="27.6" customHeight="1">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" ht="27" customHeight="1">
       <c r="B67" s="13" t="s">
         <v>23</v>
       </c>
       <c r="C67" s="12" t="s">
         <v>26</v>
       </c>
+      <c r="H67" s="1"/>
       <c r="I67" s="9" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" ht="27.6" customHeight="1">
+      <c r="B68" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="C68" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="I68" s="9" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" ht="28.2" customHeight="1">
+      <c r="A69" s="1"/>
+      <c r="B69" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C69" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="I69" s="10" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" ht="13.5" customHeight="1">
+      <c r="I70" s="6" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="68" spans="1:10" ht="28.2" customHeight="1">
-      <c r="A68" s="1"/>
-      <c r="B68" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="C68" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="I68" s="10" t="s">
+    <row r="71" spans="1:10" ht="27.6" customHeight="1">
+      <c r="I71" s="10" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="69" spans="1:10" ht="13.5" customHeight="1">
-      <c r="I69" s="6" t="s">
+    <row r="72" spans="1:10" ht="27.6" customHeight="1">
+      <c r="I72" s="9" t="s">
         <v>88</v>
-      </c>
-    </row>
-    <row r="70" spans="1:10" ht="27.6" customHeight="1">
-      <c r="I70" s="10" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="71" spans="1:10" ht="27.6" customHeight="1">
-      <c r="I71" s="9" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="72" spans="1:10" ht="13.5" customHeight="1">
-      <c r="A72" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B72" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="I72" s="8" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="73" spans="1:10" ht="13.5" customHeight="1">
       <c r="A73" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B73" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="C73" s="1"/>
-      <c r="I73" s="6" t="s">
-        <v>92</v>
+      <c r="B73" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="I73" s="8" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="74" spans="1:10" ht="13.5" customHeight="1">
       <c r="A74" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="B74" s="1"/>
+        <v>46</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>94</v>
+      </c>
       <c r="C74" s="1"/>
-      <c r="I74" s="6"/>
-    </row>
-    <row r="75" spans="1:10" ht="27.6" customHeight="1">
-      <c r="B75" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="C75" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="I75" s="9" t="s">
+      <c r="I74" s="6" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10" ht="13.5" customHeight="1">
+      <c r="A75" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="J75" s="1"/>
-    </row>
-    <row r="76" spans="1:10" ht="27" customHeight="1">
+      <c r="B75" s="1"/>
+      <c r="C75" s="1"/>
+      <c r="I75" s="6"/>
+    </row>
+    <row r="76" spans="1:10" ht="27.6" customHeight="1">
       <c r="B76" s="12" t="s">
         <v>24</v>
       </c>
@@ -2159,36 +2164,35 @@
         <v>26</v>
       </c>
       <c r="I76" s="9" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="77" spans="1:10" ht="13.5" customHeight="1">
-      <c r="A77" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="B77" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="I77" s="6"/>
+        <v>91</v>
+      </c>
+      <c r="J76" s="1"/>
+    </row>
+    <row r="77" spans="1:10" ht="27" customHeight="1">
+      <c r="B77" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C77" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="I77" s="9" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="78" spans="1:10" ht="13.5" customHeight="1">
       <c r="A78" s="3" t="s">
-        <v>96</v>
+        <v>61</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>95</v>
       </c>
       <c r="I78" s="6"/>
     </row>
     <row r="79" spans="1:10" ht="13.5" customHeight="1">
-      <c r="A79" s="1"/>
-      <c r="B79" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="C79" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="I79" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="J79" s="1"/>
+      <c r="A79" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="I79" s="6"/>
     </row>
     <row r="80" spans="1:10" ht="13.5" customHeight="1">
       <c r="A80" s="1"/>
@@ -2199,201 +2203,211 @@
         <v>26</v>
       </c>
       <c r="I80" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="J80" s="1"/>
+    </row>
+    <row r="81" spans="1:10" ht="13.5" customHeight="1">
+      <c r="A81" s="1"/>
+      <c r="B81" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C81" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="I81" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="J81" s="1"/>
+    </row>
+    <row r="82" spans="1:10" ht="13.5" customHeight="1">
+      <c r="A82" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B82" s="12" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="83" spans="1:10" ht="13.5" customHeight="1">
+      <c r="A83" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B83" s="1"/>
+      <c r="C83" s="1"/>
+      <c r="I83" s="6"/>
+    </row>
+    <row r="84" spans="1:10" ht="27" customHeight="1">
+      <c r="B84" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C84" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="I84" s="9" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="85" spans="1:10" ht="27.6" customHeight="1">
+      <c r="B85" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C85" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="I85" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="J80" s="1"/>
-    </row>
-    <row r="81" spans="1:9" ht="13.5" customHeight="1">
-      <c r="A81" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="B81" s="12" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="82" spans="1:9" ht="13.5" customHeight="1">
-      <c r="A82" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="B82" s="1"/>
-      <c r="C82" s="1"/>
-      <c r="I82" s="6"/>
-    </row>
-    <row r="83" spans="1:9" ht="27" customHeight="1">
-      <c r="B83" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="C83" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="I83" s="9" t="s">
+    </row>
+    <row r="86" spans="1:10" ht="13.5" customHeight="1">
+      <c r="B86" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C86" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="I86" s="6" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="84" spans="1:9" ht="27.6" customHeight="1">
-      <c r="B84" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="C84" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="I84" s="9" t="s">
+    <row r="87" spans="1:10" ht="13.5" customHeight="1">
+      <c r="A87" s="1"/>
+      <c r="B87" s="1"/>
+      <c r="I87" s="8" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="85" spans="1:9" ht="13.5" customHeight="1">
-      <c r="B85" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="C85" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="I85" s="6" t="s">
+    <row r="88" spans="1:10" ht="28.2" customHeight="1">
+      <c r="A88" s="1"/>
+      <c r="I88" s="10" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="86" spans="1:9" ht="13.5" customHeight="1">
-      <c r="A86" s="1"/>
-      <c r="B86" s="1"/>
-      <c r="I86" s="8" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="87" spans="1:9" ht="28.2" customHeight="1">
-      <c r="A87" s="1"/>
-      <c r="I87" s="10" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="88" spans="1:9" ht="27.6" customHeight="1">
-      <c r="B88" s="1"/>
-      <c r="C88" s="1"/>
-      <c r="I88" s="9" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="89" spans="1:9" ht="13.5" customHeight="1">
+    <row r="89" spans="1:10" ht="27.6" customHeight="1">
       <c r="B89" s="1"/>
       <c r="C89" s="1"/>
-      <c r="I89" s="6" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="90" spans="1:9" ht="28.2" customHeight="1">
+      <c r="I89" s="9" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10" ht="13.5" customHeight="1">
       <c r="B90" s="1"/>
       <c r="C90" s="1"/>
-      <c r="I90" s="9" t="s">
+      <c r="I90" s="6" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="91" spans="1:10" ht="28.2" customHeight="1">
+      <c r="B91" s="1"/>
+      <c r="C91" s="1"/>
+      <c r="I91" s="9" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10" ht="28.8" customHeight="1">
+      <c r="B92" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C92" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="I92" s="9" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="93" spans="1:10" ht="27.6" customHeight="1">
+      <c r="A93" s="1"/>
+      <c r="B93" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C93" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="I93" s="10" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="91" spans="1:9" ht="28.8" customHeight="1">
-      <c r="B91" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="C91" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="I91" s="9" t="s">
+    <row r="94" spans="1:10" ht="13.5" customHeight="1">
+      <c r="A94" s="1"/>
+      <c r="I94" s="8" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="92" spans="1:9" ht="27.6" customHeight="1">
-      <c r="A92" s="1"/>
-      <c r="B92" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="C92" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="I92" s="10" t="s">
+    <row r="95" spans="1:10" ht="13.5" customHeight="1">
+      <c r="A95" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B95" s="3" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="93" spans="1:9" ht="13.5" customHeight="1">
-      <c r="A93" s="1"/>
-      <c r="I93" s="8" t="s">
+      <c r="I95" s="6" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="94" spans="1:9" ht="13.5" customHeight="1">
-      <c r="A94" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B94" s="3" t="s">
+    <row r="96" spans="1:10" ht="13.5" customHeight="1">
+      <c r="A96" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="I96" s="6"/>
+    </row>
+    <row r="97" spans="1:10" ht="27.6" customHeight="1">
+      <c r="A97" s="1"/>
+      <c r="B97" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C97" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="I97" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="I94" s="6" t="s">
+    </row>
+    <row r="98" spans="1:10" ht="28.8" customHeight="1">
+      <c r="B98" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C98" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="H98" s="1"/>
+      <c r="I98" s="9" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="95" spans="1:9" ht="13.5" customHeight="1">
-      <c r="A95" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="I95" s="6"/>
-    </row>
-    <row r="96" spans="1:9" ht="27.6" customHeight="1">
-      <c r="A96" s="1"/>
-      <c r="B96" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="C96" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="I96" s="9" t="s">
+    <row r="99" spans="1:10" ht="13.5" customHeight="1">
+      <c r="B99" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C99" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="I99" s="6" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="97" spans="1:10" ht="28.8" customHeight="1">
-      <c r="B97" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="C97" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="H97" s="1"/>
-      <c r="I97" s="9" t="s">
+    <row r="100" spans="1:10" ht="13.5" customHeight="1">
+      <c r="A100" s="3" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="98" spans="1:10" ht="13.5" customHeight="1">
-      <c r="B98" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="C98" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="I98" s="6" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="99" spans="1:10" ht="13.5" customHeight="1">
-      <c r="A99" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="B99" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="G99" s="3"/>
-      <c r="I99" s="6"/>
-    </row>
-    <row r="100" spans="1:10" ht="13.5" customHeight="1">
-      <c r="A100" s="3"/>
-      <c r="B100" s="3"/>
-      <c r="C100" s="1"/>
+      <c r="B100" s="12" t="s">
+        <v>24</v>
+      </c>
       <c r="G100" s="3"/>
       <c r="I100" s="6"/>
     </row>
     <row r="101" spans="1:10" ht="13.5" customHeight="1">
-      <c r="A101" s="1" t="s">
+      <c r="A101" s="3"/>
+      <c r="B101" s="3"/>
+      <c r="C101" s="1"/>
+      <c r="G101" s="3"/>
+      <c r="I101" s="6"/>
+    </row>
+    <row r="102" spans="1:10" ht="13.5" customHeight="1">
+      <c r="A102" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B101" s="1" t="s">
+      <c r="B102" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="I101" s="6"/>
-    </row>
-    <row r="102" spans="1:10" ht="13.5" customHeight="1">
       <c r="I102" s="6"/>
     </row>
     <row r="103" spans="1:10" ht="13.5" customHeight="1">
@@ -2403,8 +2417,6 @@
       <c r="I104" s="6"/>
     </row>
     <row r="105" spans="1:10" ht="13.5" customHeight="1">
-      <c r="B105" s="1"/>
-      <c r="C105" s="1"/>
       <c r="I105" s="6"/>
     </row>
     <row r="106" spans="1:10" ht="13.5" customHeight="1">
@@ -2428,10 +2440,9 @@
       <c r="I109" s="6"/>
     </row>
     <row r="110" spans="1:10" ht="13.5" customHeight="1">
-      <c r="A110" s="1"/>
       <c r="B110" s="1"/>
+      <c r="C110" s="1"/>
       <c r="I110" s="6"/>
-      <c r="J110" s="1"/>
     </row>
     <row r="111" spans="1:10" ht="13.5" customHeight="1">
       <c r="A111" s="1"/>
@@ -2440,25 +2451,26 @@
       <c r="J111" s="1"/>
     </row>
     <row r="112" spans="1:10" ht="13.5" customHeight="1">
+      <c r="A112" s="1"/>
+      <c r="B112" s="1"/>
       <c r="I112" s="6"/>
       <c r="J112" s="1"/>
     </row>
     <row r="113" spans="1:10" ht="13.5" customHeight="1">
-      <c r="B113" s="1"/>
-      <c r="C113" s="1"/>
       <c r="I113" s="6"/>
+      <c r="J113" s="1"/>
     </row>
     <row r="114" spans="1:10" ht="13.5" customHeight="1">
-      <c r="A114" s="1"/>
       <c r="B114" s="1"/>
+      <c r="C114" s="1"/>
+      <c r="I114" s="6"/>
     </row>
     <row r="115" spans="1:10" ht="13.5" customHeight="1">
       <c r="A115" s="1"/>
+      <c r="B115" s="1"/>
     </row>
     <row r="116" spans="1:10" ht="13.5" customHeight="1">
-      <c r="B116" s="1"/>
-      <c r="C116" s="1"/>
-      <c r="I116" s="6"/>
+      <c r="A116" s="1"/>
     </row>
     <row r="117" spans="1:10" ht="13.5" customHeight="1">
       <c r="B117" s="1"/>
@@ -2471,19 +2483,19 @@
       <c r="I118" s="6"/>
     </row>
     <row r="119" spans="1:10" ht="13.5" customHeight="1">
-      <c r="A119" s="1"/>
       <c r="B119" s="1"/>
+      <c r="C119" s="1"/>
+      <c r="I119" s="6"/>
     </row>
     <row r="120" spans="1:10" ht="13.5" customHeight="1">
       <c r="A120" s="1"/>
       <c r="B120" s="1"/>
-      <c r="I120" s="6"/>
-      <c r="J120" s="1"/>
     </row>
     <row r="121" spans="1:10" ht="13.5" customHeight="1">
+      <c r="A121" s="1"/>
       <c r="B121" s="1"/>
-      <c r="C121" s="1"/>
       <c r="I121" s="6"/>
+      <c r="J121" s="1"/>
     </row>
     <row r="122" spans="1:10" ht="13.5" customHeight="1">
       <c r="B122" s="1"/>
@@ -2491,33 +2503,35 @@
       <c r="I122" s="6"/>
     </row>
     <row r="123" spans="1:10" ht="13.5" customHeight="1">
-      <c r="A123" s="1"/>
       <c r="B123" s="1"/>
+      <c r="C123" s="1"/>
+      <c r="I123" s="6"/>
     </row>
     <row r="124" spans="1:10" ht="13.5" customHeight="1">
       <c r="A124" s="1"/>
+      <c r="B124" s="1"/>
     </row>
     <row r="125" spans="1:10" ht="13.5" customHeight="1">
-      <c r="I125" s="6"/>
+      <c r="A125" s="1"/>
     </row>
     <row r="126" spans="1:10" ht="13.5" customHeight="1">
-      <c r="A126" s="1"/>
+      <c r="I126" s="6"/>
     </row>
     <row r="127" spans="1:10" ht="13.5" customHeight="1">
       <c r="A127" s="1"/>
     </row>
     <row r="128" spans="1:10" ht="13.5" customHeight="1">
       <c r="A128" s="1"/>
-      <c r="B128" s="1"/>
-      <c r="H128" s="1"/>
-      <c r="I128" s="6"/>
     </row>
     <row r="129" spans="1:9" ht="13.5" customHeight="1">
       <c r="A129" s="1"/>
+      <c r="B129" s="1"/>
       <c r="H129" s="1"/>
       <c r="I129" s="6"/>
     </row>
     <row r="130" spans="1:9" ht="13.5" customHeight="1">
+      <c r="A130" s="1"/>
+      <c r="H130" s="1"/>
       <c r="I130" s="6"/>
     </row>
     <row r="131" spans="1:9" ht="13.5" customHeight="1">
@@ -2538,7 +2552,9 @@
     <row r="136" spans="1:9" ht="13.5" customHeight="1">
       <c r="I136" s="6"/>
     </row>
-    <row r="137" spans="1:9" ht="13.5" customHeight="1"/>
+    <row r="137" spans="1:9" ht="13.5" customHeight="1">
+      <c r="I137" s="6"/>
+    </row>
     <row r="138" spans="1:9" ht="13.5" customHeight="1"/>
     <row r="139" spans="1:9" ht="13.5" customHeight="1"/>
     <row r="140" spans="1:9" ht="13.5" customHeight="1"/>
@@ -3457,6 +3473,7 @@
     <row r="1053" ht="13.5" customHeight="1"/>
     <row r="1054" ht="13.5" customHeight="1"/>
     <row r="1055" ht="13.5" customHeight="1"/>
+    <row r="1056" ht="13.5" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="4"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>

</xml_diff>

<commit_message>
10/16 chapter 0106 131行まで
11日目 参加時間：２時間 計：22時間
表情差分 chapter 0106まで進行中
</commit_message>
<xml_diff>
--- a/Assets/test260903/chapter0102.xlsx
+++ b/Assets/test260903/chapter0102.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9e870389230b728a/ドキュメント/GitHub/utageTest/Assets/test260903/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="910" documentId="11_9F6694A0EEBACB1C9082A027A8BF20B2877551EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A1ED150E-3967-4D81-AC53-4C8A8A3E5C87}"/>
+  <xr:revisionPtr revIDLastSave="959" documentId="11_9F6694A0EEBACB1C9082A027A8BF20B2877551EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3A4A1BDB-3968-4677-9FA7-2873B4A3C2DA}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="855" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="123">
   <si>
     <t>Command</t>
   </si>
@@ -1065,6 +1065,23 @@
       <t>カナ</t>
     </rPh>
     <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>悲しみ</t>
+  </si>
+  <si>
+    <t>悲しみ</t>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>喜び</t>
+  </si>
+  <si>
+    <t>喜び</t>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>怒り</t>
   </si>
 </sst>
 </file>
@@ -1623,7 +1640,7 @@
         <v>24</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>26</v>
+        <v>121</v>
       </c>
       <c r="I22" s="9" t="s">
         <v>47</v>
@@ -1725,7 +1742,7 @@
         <v>24</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>26</v>
+        <v>119</v>
       </c>
       <c r="I31" s="9" t="s">
         <v>109</v>
@@ -1804,7 +1821,7 @@
         <v>24</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>26</v>
+        <v>121</v>
       </c>
       <c r="I40" s="10" t="s">
         <v>110</v>
@@ -1830,7 +1847,7 @@
         <v>24</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>26</v>
+        <v>121</v>
       </c>
       <c r="I43" s="10" t="s">
         <v>62</v>
@@ -1841,7 +1858,7 @@
         <v>24</v>
       </c>
       <c r="C44" s="12" t="s">
-        <v>26</v>
+        <v>120</v>
       </c>
       <c r="I44" s="10" t="s">
         <v>63</v>
@@ -1871,8 +1888,8 @@
       <c r="B47" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="C47" s="11" t="s">
-        <v>26</v>
+      <c r="C47" s="12" t="s">
+        <v>122</v>
       </c>
       <c r="I47" s="10" t="s">
         <v>64</v>
@@ -1915,8 +1932,8 @@
       <c r="B51" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="C51" s="11" t="s">
-        <v>26</v>
+      <c r="C51" s="12" t="s">
+        <v>120</v>
       </c>
       <c r="I51" s="9" t="s">
         <v>68</v>
@@ -1927,8 +1944,8 @@
       <c r="B52" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="C52" s="13" t="s">
-        <v>25</v>
+      <c r="C52" s="12" t="s">
+        <v>120</v>
       </c>
       <c r="I52" s="9" t="s">
         <v>69</v>
@@ -1939,8 +1956,8 @@
       <c r="B53" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="C53" s="13" t="s">
-        <v>25</v>
+      <c r="C53" s="12" t="s">
+        <v>120</v>
       </c>
       <c r="I53" s="9" t="s">
         <v>111</v>
@@ -1950,8 +1967,8 @@
       <c r="B54" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="C54" s="13" t="s">
-        <v>25</v>
+      <c r="C54" s="12" t="s">
+        <v>120</v>
       </c>
       <c r="I54" s="9" t="s">
         <v>70</v>
@@ -2030,7 +2047,7 @@
         <v>24</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>26</v>
+        <v>118</v>
       </c>
       <c r="H63" s="1"/>
       <c r="I63" s="6" t="s">
@@ -2101,7 +2118,7 @@
         <v>24</v>
       </c>
       <c r="C69" s="12" t="s">
-        <v>26</v>
+        <v>118</v>
       </c>
       <c r="I69" s="10" t="s">
         <v>113</v>
@@ -2158,7 +2175,7 @@
         <v>24</v>
       </c>
       <c r="C76" s="12" t="s">
-        <v>26</v>
+        <v>118</v>
       </c>
       <c r="I76" s="9" t="s">
         <v>115</v>
@@ -2170,7 +2187,7 @@
         <v>24</v>
       </c>
       <c r="C77" s="12" t="s">
-        <v>26</v>
+        <v>118</v>
       </c>
       <c r="I77" s="9" t="s">
         <v>88</v>
@@ -2196,8 +2213,8 @@
       <c r="B80" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="C80" s="12" t="s">
-        <v>26</v>
+      <c r="C80" s="3" t="s">
+        <v>118</v>
       </c>
       <c r="I80" s="6" t="s">
         <v>92</v>
@@ -2238,7 +2255,7 @@
         <v>24</v>
       </c>
       <c r="C84" s="12" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I84" s="9" t="s">
         <v>94</v>
@@ -2249,7 +2266,7 @@
         <v>24</v>
       </c>
       <c r="C85" s="12" t="s">
-        <v>26</v>
+        <v>120</v>
       </c>
       <c r="I85" s="9" t="s">
         <v>95</v>
@@ -2259,8 +2276,8 @@
       <c r="B86" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="C86" s="12" t="s">
-        <v>26</v>
+      <c r="C86" s="3" t="s">
+        <v>120</v>
       </c>
       <c r="I86" s="6" t="s">
         <v>96</v>
@@ -2305,7 +2322,7 @@
         <v>24</v>
       </c>
       <c r="C92" s="12" t="s">
-        <v>26</v>
+        <v>120</v>
       </c>
       <c r="I92" s="9" t="s">
         <v>101</v>
@@ -2325,6 +2342,12 @@
     </row>
     <row r="94" spans="1:10" ht="13.5" customHeight="1">
       <c r="A94" s="1"/>
+      <c r="B94" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C94" s="12" t="s">
+        <v>120</v>
+      </c>
       <c r="I94" s="8" t="s">
         <v>117</v>
       </c>
@@ -2352,7 +2375,7 @@
         <v>24</v>
       </c>
       <c r="C97" s="12" t="s">
-        <v>26</v>
+        <v>120</v>
       </c>
       <c r="I97" s="9" t="s">
         <v>105</v>
@@ -2363,7 +2386,7 @@
         <v>24</v>
       </c>
       <c r="C98" s="12" t="s">
-        <v>26</v>
+        <v>122</v>
       </c>
       <c r="H98" s="1"/>
       <c r="I98" s="9" t="s">
@@ -2374,8 +2397,8 @@
       <c r="B99" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="C99" s="12" t="s">
-        <v>26</v>
+      <c r="C99" s="3" t="s">
+        <v>120</v>
       </c>
       <c r="I99" s="6" t="s">
         <v>107</v>

</xml_diff>